<commit_message>
fix/ report and backfill+extract codes
</commit_message>
<xml_diff>
--- a/data/out/dataset.xlsx
+++ b/data/out/dataset.xlsx
@@ -6775,11 +6775,7 @@
         <v>10</v>
       </c>
       <c r="AD50" t="inlineStr"/>
-      <c r="AE50" t="inlineStr">
-        <is>
-          <t>متساوية</t>
-        </is>
-      </c>
+      <c r="AE50" t="inlineStr"/>
       <c r="AF50" t="inlineStr"/>
       <c r="AG50" t="inlineStr">
         <is>
@@ -55419,11 +55415,7 @@
           <t>Orouba Skyline</t>
         </is>
       </c>
-      <c r="V405" t="inlineStr">
-        <is>
-          <t>ultra lux</t>
-        </is>
-      </c>
+      <c r="V405" t="inlineStr"/>
       <c r="W405" t="inlineStr"/>
       <c r="X405" t="inlineStr"/>
       <c r="Y405" t="inlineStr"/>

</xml_diff>